<commit_message>
ODSReader: Parse numbers correctly from .ods files
https://github.com/OpenDataServices/flatten-tool/issues/343
</commit_message>
<xml_diff>
--- a/flattentool/tests/fixtures/xlsx/types.xlsx
+++ b/flattentool/tests/fixtures/xlsx/types.xlsx
@@ -20,12 +20,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t xml:space="preserve">colInt</t>
   </si>
   <si>
     <t xml:space="preserve">colFloat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">colFloatComma</t>
   </si>
   <si>
     <t xml:space="preserve">colDate</t>
@@ -38,10 +41,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="DD/MM/YY"/>
-    <numFmt numFmtId="166" formatCode="DD/MM/YY\ HH:MM"/>
+    <numFmt numFmtId="165" formatCode="#,##0.00"/>
+    <numFmt numFmtId="166" formatCode="#,###.00"/>
+    <numFmt numFmtId="167" formatCode="DD/MM/YY"/>
+    <numFmt numFmtId="168" formatCode="DD/MM/YY\ HH:MM"/>
+    <numFmt numFmtId="169" formatCode="HH:MM:SS"/>
   </numFmts>
   <fonts count="16">
     <font>
@@ -292,7 +298,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -302,6 +308,18 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -394,49 +412,19 @@
 </styleSheet>
 </file>
 
-<file path=xl/revisions/revisionHeaders.xml><?xml version="1.0" encoding="utf-8"?>
-<headers xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" guid="{2540C00B-3C0A-44DC-82CB-60D22D5A0619}">
-  <header guid="{2540C00B-3C0A-44DC-82CB-60D22D5A0619}" dateTime="2020-02-07T16:56:00.000000000Z" userName=" " r:id="rId1" minRId="1" maxRId="4" maxSheetId="2">
-    <sheetIdMap count="1">
-      <sheetId val="1"/>
-    </sheetIdMap>
-  </header>
-</headers>
-</file>
-
-<file path=xl/revisions/revisionLog1.xml><?xml version="1.0" encoding="utf-8"?>
-<revisions xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <rrc rId="1" ua="false" sId="1" eol="0" ref="E:E" action="deleteCol">
-    <rfmt sheetId="1" sqref="E:E"/>
-  </rrc>
-  <rrc rId="2" ua="false" sId="1" eol="0" ref="E:E" action="deleteCol">
-    <rfmt sheetId="1" sqref="E:E"/>
-  </rrc>
-  <rrc rId="3" ua="false" sId="1" eol="0" ref="E:E" action="deleteCol">
-    <rfmt sheetId="1" sqref="E:E"/>
-  </rrc>
-  <rrc rId="4" ua="false" sId="1" eol="0" ref="E:E" action="deleteCol">
-    <rfmt sheetId="1" sqref="E:E"/>
-  </rrc>
-</revisions>
-</file>
-
-<file path=xl/revisions/userNames.xml><?xml version="1.0" encoding="utf-8"?>
-<users xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" count="0"/>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr filterMode="false">
     <tabColor rgb="FFFFFFFF"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="3" min="1" style="0" width="11.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="13.3"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1025" min="5" style="0" width="11.52"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="4" min="1" style="0" width="11.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="13.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="13.54"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1025" min="7" style="0" width="11.52"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -452,20 +440,28 @@
       <c r="D1" s="0" t="s">
         <v>3</v>
       </c>
+      <c r="E1" s="0" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="0" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="C2" s="1" t="n">
+      <c r="B2" s="1" t="n">
+        <v>1000.2</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>1000.2</v>
+      </c>
+      <c r="D2" s="3" t="n">
         <v>43895</v>
       </c>
-      <c r="D2" s="2" t="n">
+      <c r="E2" s="4" t="n">
         <v>43868.6951388889</v>
       </c>
+      <c r="F2" s="4"/>
+      <c r="G2" s="5"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>